<commit_message>
Add metadata and characteristics extraction
</commit_message>
<xml_diff>
--- a/data/input.xlsx
+++ b/data/input.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\All\PycharmProjects\prom_ai_boost\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{10C27ADD-A153-43D4-AA88-EB5A9D21DB87}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{71261967-A2A7-4B0C-91D3-752ED1587909}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="840" yWindow="555" windowWidth="23880" windowHeight="10740" xr2:uid="{F637FCF4-2B01-4B52-AC4A-D4415C23D60B}"/>
+    <workbookView xWindow="9375" yWindow="0" windowWidth="15750" windowHeight="12570" xr2:uid="{F637FCF4-2B01-4B52-AC4A-D4415C23D60B}"/>
   </bookViews>
   <sheets>
     <sheet name="Аркуш1" sheetId="1" r:id="rId1"/>
@@ -42,22 +42,22 @@
     <t>LEN001</t>
   </si>
   <si>
-    <t>Ноутбук для работы</t>
-  </si>
-  <si>
     <t>Мышка Logitech</t>
   </si>
   <si>
     <t>LOG001</t>
   </si>
   <si>
-    <t>Беспроводная мышь</t>
-  </si>
-  <si>
     <t xml:space="preserve">Ноутбук Lenovo </t>
   </si>
   <si>
     <t>Повтор товара</t>
+  </si>
+  <si>
+    <t>Ноутбук Lenovo IdeaPad 3</t>
+  </si>
+  <si>
+    <t>Мышка Logitech M185</t>
   </si>
 </sst>
 </file>
@@ -433,7 +433,7 @@
     <col min="3" max="3" width="22.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -451,30 +451,30 @@
       <c r="B2" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="C2" s="2" t="s">
-        <v>5</v>
+      <c r="C2" t="s">
+        <v>9</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B3" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="B3" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>8</v>
+      <c r="C3" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="B4" t="s">
         <v>4</v>
       </c>
       <c r="C4" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
   </sheetData>

</xml_diff>